<commit_message>
fix(fuentes): quitar subrayado y relleno amarillo de celdas 'Supuesto propio'
Las celdas de la columna Fuente marcadas como 'Supuesto propio' seguian
en negrita, pero perdieron el subrayado y el relleno amarillo (FFF2CC).
Se actualizo tambien el texto de la fila de titulo de la hoja Fuentes
(ya no menciona 'SUBRAYADAS'). Regenerado con add_fuentes_sheet.py --apply
en los 4 escenarios, A-Xtra_Storage y las 3 plantillas de Miscellaneous.
</commit_message>
<xml_diff>
--- a/inputs/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
+++ b/inputs/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand_Projection" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Demand_Projection" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fuentes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -32721,7 +32721,7 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Fuentes de los datos de este libro. Las fuentes SUBRAYADAS son supuestos propios del equipo de modelación (no provienen de una fuente externa). Hoja informativa: el modelo no la lee.</t>
+          <t>Fuentes de los datos de este libro. Las fuentes marcadas como 'Supuesto propio' son estimaciones internas del equipo de modelación (no provienen de una fuente externa). Hoja informativa: el modelo no la lee.</t>
         </is>
       </c>
     </row>

</xml_diff>